<commit_message>
Updated missing fields in several entries
</commit_message>
<xml_diff>
--- a/paper/screening.xlsx
+++ b/paper/screening.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WL961KX\Private\MSc\Thesis\Systematic Review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEA9221B-CDC6-4153-B579-6560372AA4E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C265100-DE73-4C5A-95BF-053EE612F169}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1403,7 +1403,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2047" uniqueCount="957">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2049" uniqueCount="957">
   <si>
     <t>Hierarchical Attention Transfer Networks for Depression Assessment from Speech</t>
   </si>
@@ -4283,7 +4283,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-415]d\ mmm;@"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4340,13 +4340,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-      <charset val="238"/>
     </font>
   </fonts>
   <fills count="2">
@@ -8832,7 +8825,9 @@
       <c r="Z51" s="1" t="s">
         <v>753</v>
       </c>
-      <c r="AA51" s="1"/>
+      <c r="AA51" s="1" t="s">
+        <v>773</v>
+      </c>
       <c r="AB51" s="1" t="s">
         <v>773</v>
       </c>
@@ -12929,7 +12924,9 @@
       <c r="AA139" s="1" t="s">
         <v>773</v>
       </c>
-      <c r="AB139" s="1"/>
+      <c r="AB139" s="1" t="s">
+        <v>773</v>
+      </c>
       <c r="AC139" s="1" t="s">
         <v>773</v>
       </c>

</xml_diff>